<commit_message>
miami point fix and power rankings fix
</commit_message>
<xml_diff>
--- a/the_alternative_f1/The_Alternative_F1.xlsx
+++ b/the_alternative_f1/The_Alternative_F1.xlsx
@@ -1756,11 +1756,11 @@
     <xf borderId="0" fillId="7" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
+    <xf borderId="7" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
     <xf borderId="14" fillId="8" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="right" vertical="bottom"/>
-    </xf>
-    <xf borderId="7" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment vertical="bottom"/>
     </xf>
     <xf borderId="14" fillId="8" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="right" vertical="bottom"/>
@@ -1889,11 +1889,11 @@
     <xf borderId="16" fillId="7" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
+    <xf borderId="15" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
     <xf borderId="17" fillId="8" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="right" vertical="bottom"/>
-    </xf>
-    <xf borderId="15" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment vertical="bottom"/>
     </xf>
     <xf borderId="17" fillId="8" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="right" vertical="bottom"/>
@@ -3437,8 +3437,8 @@
         <v>129</v>
       </c>
       <c r="AA2" s="85">
-        <f>IFERROR((VLOOKUP(T2,Scoring!$A:$B,2,0))+IF(W2="y",1,0)+IF(X2="y",1,0)+IF(Y2="y",1,0)+IF(Z2="y",1,0),0)</f>
-        <v>18</v>
+        <f>IFERROR((VLOOKUP(T2,Scoring!$D:$E,2,0))+IF(W2="y",1,0)+IF(X2="y",1,0)+IF(Y2="y",1,0)+IF(Z2="y",1,0),0)</f>
+        <v>7</v>
       </c>
       <c r="AB2" s="16">
         <v>2.0</v>
@@ -3846,8 +3846,8 @@
       <c r="Z3" s="102" t="s">
         <v>129</v>
       </c>
-      <c r="AA3" s="103">
-        <f>IFERROR((VLOOKUP(T3,Scoring!$A:$B,2,0))+IF(W3="y",1,0)+IF(X3="y",1,0)+IF(Y3="y",1,0)+IF(Z3="y",1,0),0)</f>
+      <c r="AA3" s="85">
+        <f>IFERROR((VLOOKUP(T3,Scoring!$D:$E,2,0))+IF(W3="y",1,0)+IF(X3="y",1,0)+IF(Y3="y",1,0)+IF(Z3="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AB3" s="24">
@@ -3892,7 +3892,7 @@
         <f>IFERROR((VLOOKUP(AJ3,Scoring!$A:$B,2,0))+IF(AM3="y",1,0)+IF(AN3="y",1,0)+IF(AO3="y",1,0)+IF(AP3="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="AR3" s="104"/>
+      <c r="AR3" s="103"/>
       <c r="AS3" s="98"/>
       <c r="AT3" s="98"/>
       <c r="AU3" s="99" t="s">
@@ -3907,7 +3907,7 @@
       <c r="AX3" s="102" t="s">
         <v>129</v>
       </c>
-      <c r="AY3" s="103">
+      <c r="AY3" s="104">
         <f>IFERROR((VLOOKUP(AR3,Scoring!$A:$B,2,0))+IF(AU3="y",1,0)+IF(AV3="y",1,0)+IF(AW3="y",1,0)+IF(AX3="y",1,0),0)</f>
         <v>0</v>
       </c>
@@ -3949,7 +3949,7 @@
         <f>IFERROR((VLOOKUP(BH3,Scoring!$A:$B,2,0))+IF(BK3="y",1,0)+IF(BL3="y",1,0)+IF(BM3="y",1,0)+IF(BN3="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="BP3" s="104"/>
+      <c r="BP3" s="103"/>
       <c r="BQ3" s="98"/>
       <c r="BR3" s="98"/>
       <c r="BS3" s="99" t="s">
@@ -3964,7 +3964,7 @@
       <c r="BV3" s="102" t="s">
         <v>129</v>
       </c>
-      <c r="BW3" s="103">
+      <c r="BW3" s="104">
         <f>IFERROR((VLOOKUP(BP3,Scoring!$A:$B,2,0))+IF(BS3="y",1,0)+IF(BT3="y",1,0)+IF(BU3="y",1,0)+IF(BV3="y",1,0),0)</f>
         <v>0</v>
       </c>
@@ -4025,7 +4025,7 @@
         <f>IFERROR((VLOOKUP(CN3,Scoring!$A:$B,2,0))+IF(CQ3="y",1,0)+IF(CR3="y",1,0)+IF(CS3="y",1,0)+IF(CT3="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="CV3" s="104"/>
+      <c r="CV3" s="103"/>
       <c r="CW3" s="98"/>
       <c r="CX3" s="98"/>
       <c r="CY3" s="99" t="s">
@@ -4040,7 +4040,7 @@
       <c r="DB3" s="102" t="s">
         <v>129</v>
       </c>
-      <c r="DC3" s="103">
+      <c r="DC3" s="104">
         <f>IFERROR((VLOOKUP(CV3,Scoring!$A:$B,2,0))+IF(CY3="y",1,0)+IF(CZ3="y",1,0)+IF(DA3="y",1,0)+IF(DB3="y",1,0),0)</f>
         <v>0</v>
       </c>
@@ -4082,7 +4082,7 @@
         <f>IFERROR((VLOOKUP(DL3,Scoring!$A:$B,2,0))+IF(DO3="y",1,0)+IF(DP3="y",1,0)+IF(DQ3="y",1,0)+IF(DR3="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="DT3" s="104"/>
+      <c r="DT3" s="103"/>
       <c r="DU3" s="98"/>
       <c r="DV3" s="98"/>
       <c r="DW3" s="99" t="s">
@@ -4257,8 +4257,8 @@
         <v>129</v>
       </c>
       <c r="AA4" s="85">
-        <f>IFERROR((VLOOKUP(T4,Scoring!$A:$B,2,0))+IF(W4="y",1,0)+IF(X4="y",1,0)+IF(Y4="y",1,0)+IF(Z4="y",1,0),0)</f>
-        <v>6</v>
+        <f>IFERROR((VLOOKUP(T4,Scoring!$D:$E,2,0))+IF(W4="y",1,0)+IF(X4="y",1,0)+IF(Y4="y",1,0)+IF(Z4="y",1,0),0)</f>
+        <v>2</v>
       </c>
       <c r="AB4" s="36">
         <v>3.0</v>
@@ -4670,9 +4670,9 @@
       <c r="Z5" s="132" t="s">
         <v>129</v>
       </c>
-      <c r="AA5" s="103">
-        <f>IFERROR((VLOOKUP(T5,Scoring!$A:$B,2,0))+IF(W5="y",1,0)+IF(X5="y",1,0)+IF(Y5="y",1,0)+IF(Z5="y",1,0),0)</f>
-        <v>8</v>
+      <c r="AA5" s="85">
+        <f>IFERROR((VLOOKUP(T5,Scoring!$D:$E,2,0))+IF(W5="y",1,0)+IF(X5="y",1,0)+IF(Y5="y",1,0)+IF(Z5="y",1,0),0)</f>
+        <v>3</v>
       </c>
       <c r="AB5" s="48">
         <v>23.0</v>
@@ -4731,7 +4731,7 @@
       <c r="AX5" s="132" t="s">
         <v>129</v>
       </c>
-      <c r="AY5" s="103">
+      <c r="AY5" s="104">
         <f>IFERROR((VLOOKUP(AR5,Scoring!$A:$B,2,0))+IF(AU5="y",1,0)+IF(AV5="y",1,0)+IF(AW5="y",1,0)+IF(AX5="y",1,0),0)</f>
         <v>0</v>
       </c>
@@ -4788,7 +4788,7 @@
       <c r="BV5" s="132" t="s">
         <v>129</v>
       </c>
-      <c r="BW5" s="103">
+      <c r="BW5" s="104">
         <f>IFERROR((VLOOKUP(BP5,Scoring!$A:$B,2,0))+IF(BS5="y",1,0)+IF(BT5="y",1,0)+IF(BU5="y",1,0)+IF(BV5="y",1,0),0)</f>
         <v>0</v>
       </c>
@@ -4864,7 +4864,7 @@
       <c r="DB5" s="132" t="s">
         <v>129</v>
       </c>
-      <c r="DC5" s="103">
+      <c r="DC5" s="104">
         <f>IFERROR((VLOOKUP(CV5,Scoring!$A:$B,2,0))+IF(CY5="y",1,0)+IF(CZ5="y",1,0)+IF(DA5="y",1,0)+IF(DB5="y",1,0),0)</f>
         <v>0</v>
       </c>
@@ -5081,8 +5081,8 @@
         <v>129</v>
       </c>
       <c r="AA6" s="85">
-        <f>IFERROR((VLOOKUP(T6,Scoring!$A:$B,2,0))+IF(W6="y",1,0)+IF(X6="y",1,0)+IF(Y6="y",1,0)+IF(Z6="y",1,0),0)</f>
-        <v>12</v>
+        <f>IFERROR((VLOOKUP(T6,Scoring!$D:$E,2,0))+IF(W6="y",1,0)+IF(X6="y",1,0)+IF(Y6="y",1,0)+IF(Z6="y",1,0),0)</f>
+        <v>5</v>
       </c>
       <c r="AB6" s="24">
         <v>4.0</v>
@@ -5126,7 +5126,7 @@
         <f>IFERROR((VLOOKUP(AJ6,Scoring!$A:$B,2,0))+IF(AM6="y",1,0)+IF(AN6="y",1,0)+IF(AO6="y",1,0)+IF(AP6="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="AR6" s="104"/>
+      <c r="AR6" s="103"/>
       <c r="AS6" s="98"/>
       <c r="AT6" s="98"/>
       <c r="AU6" s="99" t="s">
@@ -5183,7 +5183,7 @@
         <f>IFERROR((VLOOKUP(BH6,Scoring!$A:$B,2,0))+IF(BK6="y",1,0)+IF(BL6="y",1,0)+IF(BM6="y",1,0)+IF(BN6="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="BP6" s="104"/>
+      <c r="BP6" s="103"/>
       <c r="BQ6" s="98"/>
       <c r="BR6" s="98"/>
       <c r="BS6" s="99" t="s">
@@ -5259,7 +5259,7 @@
         <f>IFERROR((VLOOKUP(CN6,Scoring!$A:$B,2,0))+IF(CQ6="y",1,0)+IF(CR6="y",1,0)+IF(CS6="y",1,0)+IF(CT6="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="CV6" s="104"/>
+      <c r="CV6" s="103"/>
       <c r="CW6" s="98"/>
       <c r="CX6" s="98"/>
       <c r="CY6" s="99" t="s">
@@ -5316,7 +5316,7 @@
         <f>IFERROR((VLOOKUP(DL6,Scoring!$A:$B,2,0))+IF(DO6="y",1,0)+IF(DP6="y",1,0)+IF(DQ6="y",1,0)+IF(DR6="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="DT6" s="104"/>
+      <c r="DT6" s="103"/>
       <c r="DU6" s="98"/>
       <c r="DV6" s="98"/>
       <c r="DW6" s="99" t="s">
@@ -5490,9 +5490,9 @@
       <c r="Z7" s="102" t="s">
         <v>129</v>
       </c>
-      <c r="AA7" s="103">
-        <f>IFERROR((VLOOKUP(T7,Scoring!$A:$B,2,0))+IF(W7="y",1,0)+IF(X7="y",1,0)+IF(Y7="y",1,0)+IF(Z7="y",1,0),0)</f>
-        <v>15</v>
+      <c r="AA7" s="85">
+        <f>IFERROR((VLOOKUP(T7,Scoring!$D:$E,2,0))+IF(W7="y",1,0)+IF(X7="y",1,0)+IF(Y7="y",1,0)+IF(Z7="y",1,0),0)</f>
+        <v>6</v>
       </c>
       <c r="AB7" s="24">
         <v>6.0</v>
@@ -5536,7 +5536,7 @@
         <f>IFERROR((VLOOKUP(AJ7,Scoring!$A:$B,2,0))+IF(AM7="y",1,0)+IF(AN7="y",1,0)+IF(AO7="y",1,0)+IF(AP7="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="AR7" s="104"/>
+      <c r="AR7" s="103"/>
       <c r="AS7" s="98"/>
       <c r="AT7" s="98"/>
       <c r="AU7" s="99" t="s">
@@ -5551,7 +5551,7 @@
       <c r="AX7" s="102" t="s">
         <v>129</v>
       </c>
-      <c r="AY7" s="103">
+      <c r="AY7" s="104">
         <f>IFERROR((VLOOKUP(AR7,Scoring!$A:$B,2,0))+IF(AU7="y",1,0)+IF(AV7="y",1,0)+IF(AW7="y",1,0)+IF(AX7="y",1,0),0)</f>
         <v>0</v>
       </c>
@@ -5593,7 +5593,7 @@
         <f>IFERROR((VLOOKUP(BH7,Scoring!$A:$B,2,0))+IF(BK7="y",1,0)+IF(BL7="y",1,0)+IF(BM7="y",1,0)+IF(BN7="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="BP7" s="104"/>
+      <c r="BP7" s="103"/>
       <c r="BQ7" s="98"/>
       <c r="BR7" s="98"/>
       <c r="BS7" s="99" t="s">
@@ -5608,7 +5608,7 @@
       <c r="BV7" s="102" t="s">
         <v>129</v>
       </c>
-      <c r="BW7" s="103">
+      <c r="BW7" s="104">
         <f>IFERROR((VLOOKUP(BP7,Scoring!$A:$B,2,0))+IF(BS7="y",1,0)+IF(BT7="y",1,0)+IF(BU7="y",1,0)+IF(BV7="y",1,0),0)</f>
         <v>0</v>
       </c>
@@ -5669,7 +5669,7 @@
         <f>IFERROR((VLOOKUP(CN7,Scoring!$A:$B,2,0))+IF(CQ7="y",1,0)+IF(CR7="y",1,0)+IF(CS7="y",1,0)+IF(CT7="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="CV7" s="104"/>
+      <c r="CV7" s="103"/>
       <c r="CW7" s="98"/>
       <c r="CX7" s="98"/>
       <c r="CY7" s="99" t="s">
@@ -5684,7 +5684,7 @@
       <c r="DB7" s="102" t="s">
         <v>129</v>
       </c>
-      <c r="DC7" s="103">
+      <c r="DC7" s="104">
         <f>IFERROR((VLOOKUP(CV7,Scoring!$A:$B,2,0))+IF(CY7="y",1,0)+IF(CZ7="y",1,0)+IF(DA7="y",1,0)+IF(DB7="y",1,0),0)</f>
         <v>0</v>
       </c>
@@ -5726,7 +5726,7 @@
         <f>IFERROR((VLOOKUP(DL7,Scoring!$A:$B,2,0))+IF(DO7="y",1,0)+IF(DP7="y",1,0)+IF(DQ7="y",1,0)+IF(DR7="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="DT7" s="104"/>
+      <c r="DT7" s="103"/>
       <c r="DU7" s="98"/>
       <c r="DV7" s="98"/>
       <c r="DW7" s="99" t="s">
@@ -5901,8 +5901,8 @@
         <v>129</v>
       </c>
       <c r="AA8" s="85">
-        <f>IFERROR((VLOOKUP(T8,Scoring!$A:$B,2,0))+IF(W8="y",1,0)+IF(X8="y",1,0)+IF(Y8="y",1,0)+IF(Z8="y",1,0),0)</f>
-        <v>2</v>
+        <f>IFERROR((VLOOKUP(T8,Scoring!$D:$E,2,0))+IF(W8="y",1,0)+IF(X8="y",1,0)+IF(Y8="y",1,0)+IF(Z8="y",1,0),0)</f>
+        <v>0.5</v>
       </c>
       <c r="AB8" s="36">
         <v>8.0</v>
@@ -6310,9 +6310,9 @@
       <c r="Z9" s="132" t="s">
         <v>129</v>
       </c>
-      <c r="AA9" s="103">
-        <f>IFERROR((VLOOKUP(T9,Scoring!$A:$B,2,0))+IF(W9="y",1,0)+IF(X9="y",1,0)+IF(Y9="y",1,0)+IF(Z9="y",1,0),0)</f>
-        <v>3</v>
+      <c r="AA9" s="85">
+        <f>IFERROR((VLOOKUP(T9,Scoring!$D:$E,2,0))+IF(W9="y",1,0)+IF(X9="y",1,0)+IF(Y9="y",1,0)+IF(Z9="y",1,0),0)</f>
+        <v>0.5</v>
       </c>
       <c r="AB9" s="48">
         <v>23.0</v>
@@ -6371,7 +6371,7 @@
       <c r="AX9" s="132" t="s">
         <v>129</v>
       </c>
-      <c r="AY9" s="103">
+      <c r="AY9" s="104">
         <f>IFERROR((VLOOKUP(AR9,Scoring!$A:$B,2,0))+IF(AU9="y",1,0)+IF(AV9="y",1,0)+IF(AW9="y",1,0)+IF(AX9="y",1,0),0)</f>
         <v>0</v>
       </c>
@@ -6428,7 +6428,7 @@
       <c r="BV9" s="132" t="s">
         <v>129</v>
       </c>
-      <c r="BW9" s="103">
+      <c r="BW9" s="104">
         <f>IFERROR((VLOOKUP(BP9,Scoring!$A:$B,2,0))+IF(BS9="y",1,0)+IF(BT9="y",1,0)+IF(BU9="y",1,0)+IF(BV9="y",1,0),0)</f>
         <v>0</v>
       </c>
@@ -6504,7 +6504,7 @@
       <c r="DB9" s="132" t="s">
         <v>129</v>
       </c>
-      <c r="DC9" s="103">
+      <c r="DC9" s="104">
         <f>IFERROR((VLOOKUP(CV9,Scoring!$A:$B,2,0))+IF(CY9="y",1,0)+IF(CZ9="y",1,0)+IF(DA9="y",1,0)+IF(DB9="y",1,0),0)</f>
         <v>0</v>
       </c>
@@ -6721,7 +6721,7 @@
         <v>129</v>
       </c>
       <c r="AA10" s="85">
-        <f>IFERROR((VLOOKUP(T10,Scoring!$A:$B,2,0))+IF(W10="y",1,0)+IF(X10="y",1,0)+IF(Y10="y",1,0)+IF(Z10="y",1,0),0)</f>
+        <f>IFERROR((VLOOKUP(T10,Scoring!$D:$E,2,0))+IF(W10="y",1,0)+IF(X10="y",1,0)+IF(Y10="y",1,0)+IF(Z10="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AB10" s="24">
@@ -6766,7 +6766,7 @@
         <f>IFERROR((VLOOKUP(AJ10,Scoring!$A:$B,2,0))+IF(AM10="y",1,0)+IF(AN10="y",1,0)+IF(AO10="y",1,0)+IF(AP10="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="AR10" s="104"/>
+      <c r="AR10" s="103"/>
       <c r="AS10" s="98"/>
       <c r="AT10" s="98"/>
       <c r="AU10" s="99" t="s">
@@ -6823,7 +6823,7 @@
         <f>IFERROR((VLOOKUP(BH10,Scoring!$A:$B,2,0))+IF(BK10="y",1,0)+IF(BL10="y",1,0)+IF(BM10="y",1,0)+IF(BN10="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="BP10" s="104"/>
+      <c r="BP10" s="103"/>
       <c r="BQ10" s="98"/>
       <c r="BR10" s="98"/>
       <c r="BS10" s="99" t="s">
@@ -6899,7 +6899,7 @@
         <f>IFERROR((VLOOKUP(CN10,Scoring!$A:$B,2,0))+IF(CQ10="y",1,0)+IF(CR10="y",1,0)+IF(CS10="y",1,0)+IF(CT10="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="CV10" s="104"/>
+      <c r="CV10" s="103"/>
       <c r="CW10" s="98"/>
       <c r="CX10" s="98"/>
       <c r="CY10" s="99" t="s">
@@ -6956,7 +6956,7 @@
         <f>IFERROR((VLOOKUP(DL10,Scoring!$A:$B,2,0))+IF(DO10="y",1,0)+IF(DP10="y",1,0)+IF(DQ10="y",1,0)+IF(DR10="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="DT10" s="104"/>
+      <c r="DT10" s="103"/>
       <c r="DU10" s="98"/>
       <c r="DV10" s="98"/>
       <c r="DW10" s="99" t="s">
@@ -7130,8 +7130,8 @@
       <c r="Z11" s="102" t="s">
         <v>129</v>
       </c>
-      <c r="AA11" s="103">
-        <f>IFERROR((VLOOKUP(T11,Scoring!$A:$B,2,0))+IF(W11="y",1,0)+IF(X11="y",1,0)+IF(Y11="y",1,0)+IF(Z11="y",1,0),0)</f>
+      <c r="AA11" s="85">
+        <f>IFERROR((VLOOKUP(T11,Scoring!$D:$E,2,0))+IF(W11="y",1,0)+IF(X11="y",1,0)+IF(Y11="y",1,0)+IF(Z11="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AB11" s="24">
@@ -7176,7 +7176,7 @@
         <f>IFERROR((VLOOKUP(AJ11,Scoring!$A:$B,2,0))+IF(AM11="y",1,0)+IF(AN11="y",1,0)+IF(AO11="y",1,0)+IF(AP11="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="AR11" s="104"/>
+      <c r="AR11" s="103"/>
       <c r="AS11" s="98"/>
       <c r="AT11" s="98"/>
       <c r="AU11" s="99" t="s">
@@ -7191,7 +7191,7 @@
       <c r="AX11" s="102" t="s">
         <v>129</v>
       </c>
-      <c r="AY11" s="103">
+      <c r="AY11" s="104">
         <f>IFERROR((VLOOKUP(AR11,Scoring!$A:$B,2,0))+IF(AU11="y",1,0)+IF(AV11="y",1,0)+IF(AW11="y",1,0)+IF(AX11="y",1,0),0)</f>
         <v>0</v>
       </c>
@@ -7233,7 +7233,7 @@
         <f>IFERROR((VLOOKUP(BH11,Scoring!$A:$B,2,0))+IF(BK11="y",1,0)+IF(BL11="y",1,0)+IF(BM11="y",1,0)+IF(BN11="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="BP11" s="104"/>
+      <c r="BP11" s="103"/>
       <c r="BQ11" s="98"/>
       <c r="BR11" s="98"/>
       <c r="BS11" s="99" t="s">
@@ -7248,7 +7248,7 @@
       <c r="BV11" s="102" t="s">
         <v>129</v>
       </c>
-      <c r="BW11" s="103">
+      <c r="BW11" s="104">
         <f>IFERROR((VLOOKUP(BP11,Scoring!$A:$B,2,0))+IF(BS11="y",1,0)+IF(BT11="y",1,0)+IF(BU11="y",1,0)+IF(BV11="y",1,0),0)</f>
         <v>0</v>
       </c>
@@ -7309,7 +7309,7 @@
         <f>IFERROR((VLOOKUP(CN11,Scoring!$A:$B,2,0))+IF(CQ11="y",1,0)+IF(CR11="y",1,0)+IF(CS11="y",1,0)+IF(CT11="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="CV11" s="104"/>
+      <c r="CV11" s="103"/>
       <c r="CW11" s="98"/>
       <c r="CX11" s="98"/>
       <c r="CY11" s="99" t="s">
@@ -7324,7 +7324,7 @@
       <c r="DB11" s="102" t="s">
         <v>129</v>
       </c>
-      <c r="DC11" s="103">
+      <c r="DC11" s="104">
         <f>IFERROR((VLOOKUP(CV11,Scoring!$A:$B,2,0))+IF(CY11="y",1,0)+IF(CZ11="y",1,0)+IF(DA11="y",1,0)+IF(DB11="y",1,0),0)</f>
         <v>0</v>
       </c>
@@ -7366,7 +7366,7 @@
         <f>IFERROR((VLOOKUP(DL11,Scoring!$A:$B,2,0))+IF(DO11="y",1,0)+IF(DP11="y",1,0)+IF(DQ11="y",1,0)+IF(DR11="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="DT11" s="104"/>
+      <c r="DT11" s="103"/>
       <c r="DU11" s="98"/>
       <c r="DV11" s="98"/>
       <c r="DW11" s="99" t="s">
@@ -7541,7 +7541,7 @@
         <v>129</v>
       </c>
       <c r="AA12" s="85">
-        <f>IFERROR((VLOOKUP(T12,Scoring!$A:$B,2,0))+IF(W12="y",1,0)+IF(X12="y",1,0)+IF(Y12="y",1,0)+IF(Z12="y",1,0),0)</f>
+        <f>IFERROR((VLOOKUP(T12,Scoring!$D:$E,2,0))+IF(W12="y",1,0)+IF(X12="y",1,0)+IF(Y12="y",1,0)+IF(Z12="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AB12" s="36">
@@ -7950,8 +7950,8 @@
       <c r="Z13" s="102" t="s">
         <v>129</v>
       </c>
-      <c r="AA13" s="103">
-        <f>IFERROR((VLOOKUP(T13,Scoring!$A:$B,2,0))+IF(W13="y",1,0)+IF(X13="y",1,0)+IF(Y13="y",1,0)+IF(Z13="y",1,0),0)</f>
+      <c r="AA13" s="85">
+        <f>IFERROR((VLOOKUP(T13,Scoring!$D:$E,2,0))+IF(W13="y",1,0)+IF(X13="y",1,0)+IF(Y13="y",1,0)+IF(Z13="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AB13" s="24">
@@ -7996,7 +7996,7 @@
         <f>IFERROR((VLOOKUP(AJ13,Scoring!$A:$B,2,0))+IF(AM13="y",1,0)+IF(AN13="y",1,0)+IF(AO13="y",1,0)+IF(AP13="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="AR13" s="104"/>
+      <c r="AR13" s="103"/>
       <c r="AS13" s="98"/>
       <c r="AT13" s="98"/>
       <c r="AU13" s="99" t="s">
@@ -8011,7 +8011,7 @@
       <c r="AX13" s="102" t="s">
         <v>129</v>
       </c>
-      <c r="AY13" s="103">
+      <c r="AY13" s="104">
         <f>IFERROR((VLOOKUP(AR13,Scoring!$A:$B,2,0))+IF(AU13="y",1,0)+IF(AV13="y",1,0)+IF(AW13="y",1,0)+IF(AX13="y",1,0),0)</f>
         <v>0</v>
       </c>
@@ -8053,7 +8053,7 @@
         <f>IFERROR((VLOOKUP(BH13,Scoring!$A:$B,2,0))+IF(BK13="y",1,0)+IF(BL13="y",1,0)+IF(BM13="y",1,0)+IF(BN13="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="BP13" s="104"/>
+      <c r="BP13" s="103"/>
       <c r="BQ13" s="98"/>
       <c r="BR13" s="98"/>
       <c r="BS13" s="99" t="s">
@@ -8068,7 +8068,7 @@
       <c r="BV13" s="102" t="s">
         <v>129</v>
       </c>
-      <c r="BW13" s="103">
+      <c r="BW13" s="104">
         <f>IFERROR((VLOOKUP(BP13,Scoring!$A:$B,2,0))+IF(BS13="y",1,0)+IF(BT13="y",1,0)+IF(BU13="y",1,0)+IF(BV13="y",1,0),0)</f>
         <v>0</v>
       </c>
@@ -8129,7 +8129,7 @@
         <f>IFERROR((VLOOKUP(CN13,Scoring!$A:$B,2,0))+IF(CQ13="y",1,0)+IF(CR13="y",1,0)+IF(CS13="y",1,0)+IF(CT13="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="CV13" s="104"/>
+      <c r="CV13" s="103"/>
       <c r="CW13" s="98"/>
       <c r="CX13" s="98"/>
       <c r="CY13" s="99" t="s">
@@ -8144,7 +8144,7 @@
       <c r="DB13" s="102" t="s">
         <v>129</v>
       </c>
-      <c r="DC13" s="103">
+      <c r="DC13" s="104">
         <f>IFERROR((VLOOKUP(CV13,Scoring!$A:$B,2,0))+IF(CY13="y",1,0)+IF(CZ13="y",1,0)+IF(DA13="y",1,0)+IF(DB13="y",1,0),0)</f>
         <v>0</v>
       </c>
@@ -8186,7 +8186,7 @@
         <f>IFERROR((VLOOKUP(DL13,Scoring!$A:$B,2,0))+IF(DO13="y",1,0)+IF(DP13="y",1,0)+IF(DQ13="y",1,0)+IF(DR13="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="DT13" s="104"/>
+      <c r="DT13" s="103"/>
       <c r="DU13" s="98"/>
       <c r="DV13" s="98"/>
       <c r="DW13" s="99" t="s">
@@ -8361,8 +8361,8 @@
         <v>129</v>
       </c>
       <c r="AA14" s="85">
-        <f>IFERROR((VLOOKUP(T14,Scoring!$A:$B,2,0))+IF(W14="y",1,0)+IF(X14="y",1,0)+IF(Y14="y",1,0)+IF(Z14="y",1,0),0)</f>
-        <v>25</v>
+        <f>IFERROR((VLOOKUP(T14,Scoring!$D:$E,2,0))+IF(W14="y",1,0)+IF(X14="y",1,0)+IF(Y14="y",1,0)+IF(Z14="y",1,0),0)</f>
+        <v>8</v>
       </c>
       <c r="AB14" s="36">
         <v>5.0</v>
@@ -8770,8 +8770,8 @@
       <c r="Z15" s="132" t="s">
         <v>129</v>
       </c>
-      <c r="AA15" s="103">
-        <f>IFERROR((VLOOKUP(T15,Scoring!$A:$B,2,0))+IF(W15="y",1,0)+IF(X15="y",1,0)+IF(Y15="y",1,0)+IF(Z15="y",1,0),0)</f>
+      <c r="AA15" s="85">
+        <f>IFERROR((VLOOKUP(T15,Scoring!$D:$E,2,0))+IF(W15="y",1,0)+IF(X15="y",1,0)+IF(Y15="y",1,0)+IF(Z15="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AB15" s="48">
@@ -8831,7 +8831,7 @@
       <c r="AX15" s="132" t="s">
         <v>129</v>
       </c>
-      <c r="AY15" s="103">
+      <c r="AY15" s="104">
         <f>IFERROR((VLOOKUP(AR15,Scoring!$A:$B,2,0))+IF(AU15="y",1,0)+IF(AV15="y",1,0)+IF(AW15="y",1,0)+IF(AX15="y",1,0),0)</f>
         <v>0</v>
       </c>
@@ -8888,7 +8888,7 @@
       <c r="BV15" s="132" t="s">
         <v>129</v>
       </c>
-      <c r="BW15" s="103">
+      <c r="BW15" s="104">
         <f>IFERROR((VLOOKUP(BP15,Scoring!$A:$B,2,0))+IF(BS15="y",1,0)+IF(BT15="y",1,0)+IF(BU15="y",1,0)+IF(BV15="y",1,0),0)</f>
         <v>0</v>
       </c>
@@ -8964,7 +8964,7 @@
       <c r="DB15" s="132" t="s">
         <v>129</v>
       </c>
-      <c r="DC15" s="103">
+      <c r="DC15" s="104">
         <f>IFERROR((VLOOKUP(CV15,Scoring!$A:$B,2,0))+IF(CY15="y",1,0)+IF(CZ15="y",1,0)+IF(DA15="y",1,0)+IF(DB15="y",1,0),0)</f>
         <v>0</v>
       </c>
@@ -9181,8 +9181,8 @@
         <v>129</v>
       </c>
       <c r="AA16" s="85">
-        <f>IFERROR((VLOOKUP(T16,Scoring!$A:$B,2,0))+IF(W16="y",1,0)+IF(X16="y",1,0)+IF(Y16="y",1,0)+IF(Z16="y",1,0),0)</f>
-        <v>10</v>
+        <f>IFERROR((VLOOKUP(T16,Scoring!$D:$E,2,0))+IF(W16="y",1,0)+IF(X16="y",1,0)+IF(Y16="y",1,0)+IF(Z16="y",1,0),0)</f>
+        <v>4</v>
       </c>
       <c r="AB16" s="24">
         <v>1.0</v>
@@ -9226,7 +9226,7 @@
         <f>IFERROR((VLOOKUP(AJ16,Scoring!$A:$B,2,0))+IF(AM16="y",1,0)+IF(AN16="y",1,0)+IF(AO16="y",1,0)+IF(AP16="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="AR16" s="104"/>
+      <c r="AR16" s="103"/>
       <c r="AS16" s="98"/>
       <c r="AT16" s="98"/>
       <c r="AU16" s="99" t="s">
@@ -9283,7 +9283,7 @@
         <f>IFERROR((VLOOKUP(BH16,Scoring!$A:$B,2,0))+IF(BK16="y",1,0)+IF(BL16="y",1,0)+IF(BM16="y",1,0)+IF(BN16="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="BP16" s="104"/>
+      <c r="BP16" s="103"/>
       <c r="BQ16" s="98"/>
       <c r="BR16" s="98"/>
       <c r="BS16" s="99" t="s">
@@ -9359,7 +9359,7 @@
         <f>IFERROR((VLOOKUP(CN16,Scoring!$A:$B,2,0))+IF(CQ16="y",1,0)+IF(CR16="y",1,0)+IF(CS16="y",1,0)+IF(CT16="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="CV16" s="104"/>
+      <c r="CV16" s="103"/>
       <c r="CW16" s="98"/>
       <c r="CX16" s="98"/>
       <c r="CY16" s="99" t="s">
@@ -9416,7 +9416,7 @@
         <f>IFERROR((VLOOKUP(DL16,Scoring!$A:$B,2,0))+IF(DO16="y",1,0)+IF(DP16="y",1,0)+IF(DQ16="y",1,0)+IF(DR16="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="DT16" s="104"/>
+      <c r="DT16" s="103"/>
       <c r="DU16" s="98"/>
       <c r="DV16" s="98"/>
       <c r="DW16" s="99" t="s">
@@ -9592,9 +9592,9 @@
       <c r="Z17" s="147" t="s">
         <v>129</v>
       </c>
-      <c r="AA17" s="148">
-        <f>IFERROR((VLOOKUP(T17,Scoring!$A:$B,2,0))+IF(W17="y",1,0)+IF(X17="y",1,0)+IF(Y17="y",1,0)+IF(Z17="y",1,0),0)</f>
-        <v>4</v>
+      <c r="AA17" s="85">
+        <f>IFERROR((VLOOKUP(T17,Scoring!$D:$E,2,0))+IF(W17="y",1,0)+IF(X17="y",1,0)+IF(Y17="y",1,0)+IF(Z17="y",1,0),0)</f>
+        <v>1</v>
       </c>
       <c r="AB17" s="60">
         <v>9.0</v>
@@ -9638,7 +9638,7 @@
         <f>IFERROR((VLOOKUP(AJ17,Scoring!$A:$B,2,0))+IF(AM17="y",1,0)+IF(AN17="y",1,0)+IF(AO17="y",1,0)+IF(AP17="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="AR17" s="149"/>
+      <c r="AR17" s="148"/>
       <c r="AS17" s="143"/>
       <c r="AT17" s="143"/>
       <c r="AU17" s="144" t="s">
@@ -9653,7 +9653,7 @@
       <c r="AX17" s="147" t="s">
         <v>129</v>
       </c>
-      <c r="AY17" s="148">
+      <c r="AY17" s="149">
         <f>IFERROR((VLOOKUP(AR17,Scoring!$A:$B,2,0))+IF(AU17="y",1,0)+IF(AV17="y",1,0)+IF(AW17="y",1,0)+IF(AX17="y",1,0),0)</f>
         <v>0</v>
       </c>
@@ -9695,7 +9695,7 @@
         <f>IFERROR((VLOOKUP(BH17,Scoring!$A:$B,2,0))+IF(BK17="y",1,0)+IF(BL17="y",1,0)+IF(BM17="y",1,0)+IF(BN17="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="BP17" s="149"/>
+      <c r="BP17" s="148"/>
       <c r="BQ17" s="143"/>
       <c r="BR17" s="143"/>
       <c r="BS17" s="144" t="s">
@@ -9710,7 +9710,7 @@
       <c r="BV17" s="147" t="s">
         <v>129</v>
       </c>
-      <c r="BW17" s="148">
+      <c r="BW17" s="149">
         <f>IFERROR((VLOOKUP(BP17,Scoring!$A:$B,2,0))+IF(BS17="y",1,0)+IF(BT17="y",1,0)+IF(BU17="y",1,0)+IF(BV17="y",1,0),0)</f>
         <v>0</v>
       </c>
@@ -9771,7 +9771,7 @@
         <f>IFERROR((VLOOKUP(CN17,Scoring!$A:$B,2,0))+IF(CQ17="y",1,0)+IF(CR17="y",1,0)+IF(CS17="y",1,0)+IF(CT17="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="CV17" s="149"/>
+      <c r="CV17" s="148"/>
       <c r="CW17" s="143"/>
       <c r="CX17" s="143"/>
       <c r="CY17" s="144" t="s">
@@ -9786,7 +9786,7 @@
       <c r="DB17" s="147" t="s">
         <v>129</v>
       </c>
-      <c r="DC17" s="148">
+      <c r="DC17" s="149">
         <f>IFERROR((VLOOKUP(CV17,Scoring!$A:$B,2,0))+IF(CY17="y",1,0)+IF(CZ17="y",1,0)+IF(DA17="y",1,0)+IF(DB17="y",1,0),0)</f>
         <v>0</v>
       </c>
@@ -9828,7 +9828,7 @@
         <f>IFERROR((VLOOKUP(DL17,Scoring!$A:$B,2,0))+IF(DO17="y",1,0)+IF(DP17="y",1,0)+IF(DQ17="y",1,0)+IF(DR17="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="DT17" s="149"/>
+      <c r="DT17" s="148"/>
       <c r="DU17" s="143"/>
       <c r="DV17" s="143"/>
       <c r="DW17" s="144" t="s">

</xml_diff>

<commit_message>
points fix, QOL for chat
</commit_message>
<xml_diff>
--- a/the_alternative_f1/The_Alternative_F1.xlsx
+++ b/the_alternative_f1/The_Alternative_F1.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3634" uniqueCount="406">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3634" uniqueCount="407">
   <si>
     <t>Positions</t>
   </si>
@@ -826,6 +826,9 @@
   </si>
   <si>
     <t>n</t>
+  </si>
+  <si>
+    <t>Jelly</t>
   </si>
   <si>
     <t>Jaden</t>
@@ -2472,18 +2475,18 @@
         <v>192</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B2" s="69" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="3">
@@ -2491,21 +2494,21 @@
         <v>142</v>
       </c>
       <c r="B3" s="69" t="s">
+        <v>275</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>274</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B4" s="69" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="5">
@@ -2513,10 +2516,10 @@
         <v>145</v>
       </c>
       <c r="B5" s="69" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="6">
@@ -2524,10 +2527,10 @@
         <v>146</v>
       </c>
       <c r="B6" s="69" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="7">
@@ -2535,10 +2538,10 @@
         <v>157</v>
       </c>
       <c r="B7" s="69" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="8">
@@ -2546,32 +2549,32 @@
         <v>195</v>
       </c>
       <c r="B8" s="69" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B9" s="69" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B10" s="69" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="11">
@@ -2579,21 +2582,21 @@
         <v>150</v>
       </c>
       <c r="B11" s="69" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B12" s="69" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="13">
@@ -2601,10 +2604,10 @@
         <v>158</v>
       </c>
       <c r="B13" s="69" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="14">
@@ -2612,10 +2615,10 @@
         <v>148</v>
       </c>
       <c r="B14" s="69" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="15">
@@ -2623,10 +2626,10 @@
         <v>151</v>
       </c>
       <c r="B15" s="69" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="16">
@@ -2634,10 +2637,10 @@
         <v>143</v>
       </c>
       <c r="B16" s="69" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="17">
@@ -2645,10 +2648,10 @@
         <v>159</v>
       </c>
       <c r="B17" s="69" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="18">
@@ -2656,10 +2659,10 @@
         <v>160</v>
       </c>
       <c r="B18" s="69" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="19">
@@ -2667,10 +2670,10 @@
         <v>152</v>
       </c>
       <c r="B19" s="69" t="s">
+        <v>292</v>
+      </c>
+      <c r="C19" s="1" t="s">
         <v>291</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>290</v>
       </c>
     </row>
     <row r="20">
@@ -2678,10 +2681,10 @@
         <v>198</v>
       </c>
       <c r="B20" s="69" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
   </sheetData>
@@ -2879,46 +2882,46 @@
         <v>61</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="G1" s="8" t="s">
         <v>62</v>
       </c>
       <c r="H1" s="9" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="J1" s="11" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="K1" s="70" t="s">
         <v>63</v>
       </c>
       <c r="L1" s="6" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="M1" s="7" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="N1" s="7" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="O1" s="8" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="P1" s="9" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="Q1" s="10" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="R1" s="11" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="S1" s="70" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="T1" s="71" t="s">
         <v>202</v>
@@ -2927,7 +2930,7 @@
         <v>203</v>
       </c>
       <c r="V1" s="72" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="W1" s="73" t="s">
         <v>204</v>
@@ -2951,7 +2954,7 @@
         <v>65</v>
       </c>
       <c r="AD1" s="7" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="AE1" s="8" t="s">
         <v>66</v>
@@ -2975,7 +2978,7 @@
         <v>93</v>
       </c>
       <c r="AL1" s="7" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="AM1" s="8" t="s">
         <v>94</v>
@@ -2999,7 +3002,7 @@
         <v>229</v>
       </c>
       <c r="AT1" s="72" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="AU1" s="73" t="s">
         <v>230</v>
@@ -3023,7 +3026,7 @@
         <v>85</v>
       </c>
       <c r="BB1" s="7" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="BC1" s="8" t="s">
         <v>86</v>
@@ -3047,7 +3050,7 @@
         <v>117</v>
       </c>
       <c r="BJ1" s="7" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="BK1" s="8" t="s">
         <v>118</v>
@@ -3065,28 +3068,28 @@
         <v>119</v>
       </c>
       <c r="BP1" s="71" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="BQ1" s="72" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="BR1" s="72" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="BS1" s="73" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="BT1" s="74" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="BU1" s="75" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="BV1" s="76" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="BW1" s="77" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="BX1" s="6" t="s">
         <v>80</v>
@@ -3095,19 +3098,19 @@
         <v>81</v>
       </c>
       <c r="BZ1" s="7" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="CA1" s="8" t="s">
         <v>82</v>
       </c>
       <c r="CB1" s="9" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="CC1" s="10" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="CD1" s="11" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="CE1" s="70" t="s">
         <v>83</v>
@@ -3119,19 +3122,19 @@
         <v>101</v>
       </c>
       <c r="CH1" s="7" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="CI1" s="8" t="s">
         <v>102</v>
       </c>
       <c r="CJ1" s="9" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="CK1" s="10" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="CL1" s="11" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="CM1" s="70" t="s">
         <v>103</v>
@@ -3143,7 +3146,7 @@
         <v>125</v>
       </c>
       <c r="CP1" s="7" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="CQ1" s="8" t="s">
         <v>126</v>
@@ -3161,28 +3164,28 @@
         <v>127</v>
       </c>
       <c r="CV1" s="71" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="CW1" s="72" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="CX1" s="72" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="CY1" s="73" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="CZ1" s="74" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="DA1" s="75" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="DB1" s="76" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="DC1" s="77" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="DD1" s="6" t="s">
         <v>52</v>
@@ -3191,7 +3194,7 @@
         <v>53</v>
       </c>
       <c r="DF1" s="7" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="DG1" s="8" t="s">
         <v>54</v>
@@ -3215,46 +3218,46 @@
         <v>109</v>
       </c>
       <c r="DN1" s="7" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="DO1" s="8" t="s">
         <v>110</v>
       </c>
       <c r="DP1" s="9" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="DQ1" s="10" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="DR1" s="11" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="DS1" s="70" t="s">
         <v>111</v>
       </c>
       <c r="DT1" s="71" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="DU1" s="72" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="DV1" s="72" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="DW1" s="73" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="DX1" s="74" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="DY1" s="75" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="DZ1" s="76" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="EA1" s="77" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="EB1" s="71" t="s">
         <v>88</v>
@@ -3263,7 +3266,7 @@
         <v>89</v>
       </c>
       <c r="ED1" s="72" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="EE1" s="73" t="s">
         <v>90</v>
@@ -3287,46 +3290,46 @@
         <v>105</v>
       </c>
       <c r="EL1" s="7" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="EM1" s="8" t="s">
         <v>106</v>
       </c>
       <c r="EN1" s="9" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="EO1" s="10" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="EP1" s="11" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="EQ1" s="70" t="s">
         <v>107</v>
       </c>
       <c r="ER1" s="71" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="ES1" s="72" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="ET1" s="72" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="EU1" s="73" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="EV1" s="74" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="EW1" s="75" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="EX1" s="76" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="EY1" s="77" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="EZ1" s="6" t="s">
         <v>96</v>
@@ -3335,19 +3338,19 @@
         <v>97</v>
       </c>
       <c r="FB1" s="7" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="FC1" s="8" t="s">
         <v>98</v>
       </c>
       <c r="FD1" s="9" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="FE1" s="10" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="FF1" s="11" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="FG1" s="70" t="s">
         <v>99</v>
@@ -3461,7 +3464,7 @@
         <v>20</v>
       </c>
       <c r="AJ2" s="16">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="AK2" s="17">
         <v>2.0</v>
@@ -3481,7 +3484,7 @@
       </c>
       <c r="AQ2" s="78">
         <f>IFERROR((VLOOKUP(AJ2,Scoring!$A:$B,2,0))+IF(AM2="y",1,0)+IF(AN2="y",1,0)+IF(AO2="y",1,0)+IF(AP2="y",1,0),0)</f>
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="AR2" s="86"/>
       <c r="AS2" s="87"/>
@@ -5024,7 +5027,7 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>23</v>
@@ -5438,10 +5441,10 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>25</v>
+        <v>268</v>
       </c>
       <c r="C7" s="15" t="s">
         <v>26</v>
@@ -5539,7 +5542,7 @@
         <v>9</v>
       </c>
       <c r="AJ7" s="24">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="AK7" s="25">
         <v>1.0</v>
@@ -5559,7 +5562,7 @@
       </c>
       <c r="AQ7" s="95">
         <f>IFERROR((VLOOKUP(AJ7,Scoring!$A:$B,2,0))+IF(AM7="y",1,0)+IF(AN7="y",1,0)+IF(AO7="y",1,0)+IF(AP7="y",1,0),0)</f>
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="AR7" s="103"/>
       <c r="AS7" s="98"/>
@@ -5852,7 +5855,7 @@
     </row>
     <row r="8">
       <c r="A8" s="33" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="B8" s="34" t="s">
         <v>28</v>
@@ -6266,7 +6269,7 @@
     </row>
     <row r="9">
       <c r="A9" s="45" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="B9" s="46" t="s">
         <v>30</v>
@@ -6680,13 +6683,13 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="D10" s="24">
         <v>15.0</v>
@@ -7094,13 +7097,13 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="D11" s="24">
         <v>13.0</v>
@@ -7508,7 +7511,7 @@
     </row>
     <row r="12">
       <c r="A12" s="33" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="B12" s="34" t="s">
         <v>35</v>
@@ -7922,13 +7925,13 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="D13" s="24">
         <v>14.0</v>
@@ -8339,7 +8342,7 @@
         <v>37</v>
       </c>
       <c r="B14" s="34" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C14" s="35" t="s">
         <v>44</v>
@@ -8437,7 +8440,7 @@
         <v>10</v>
       </c>
       <c r="AJ14" s="36">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="AK14" s="37">
         <v>6.0</v>
@@ -8457,7 +8460,7 @@
       </c>
       <c r="AQ14" s="78">
         <f>IFERROR((VLOOKUP(AJ14,Scoring!$A:$B,2,0))+IF(AM14="y",1,0)+IF(AN14="y",1,0)+IF(AO14="y",1,0)+IF(AP14="y",1,0),0)</f>
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="AR14" s="118"/>
       <c r="AS14" s="113"/>
@@ -9172,7 +9175,7 @@
         <v>45</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="D16" s="24">
         <v>3.0</v>
@@ -9583,10 +9586,10 @@
         <v>42</v>
       </c>
       <c r="B17" s="58" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C17" s="59" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="D17" s="60">
         <v>9.0</v>
@@ -10017,40 +10020,40 @@
         <v>192</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="B2" s="69" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
+        <v>383</v>
+      </c>
+      <c r="B3" s="69" t="s">
+        <v>384</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>382</v>
-      </c>
-      <c r="B3" s="69" t="s">
-        <v>383</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>381</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="B4" s="69" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
     </row>
     <row r="5">
@@ -10058,32 +10061,32 @@
         <v>144</v>
       </c>
       <c r="B5" s="69" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B6" s="69" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B7" s="69" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="8">
@@ -10091,10 +10094,10 @@
         <v>145</v>
       </c>
       <c r="B8" s="69" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="9">
@@ -10102,21 +10105,21 @@
         <v>152</v>
       </c>
       <c r="B9" s="69" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B10" s="69" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="11">
@@ -10124,10 +10127,10 @@
         <v>150</v>
       </c>
       <c r="B11" s="69" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="12">
@@ -10135,21 +10138,21 @@
         <v>158</v>
       </c>
       <c r="B12" s="69" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B13" s="69" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="14">
@@ -10157,10 +10160,10 @@
         <v>149</v>
       </c>
       <c r="B14" s="69" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="15">
@@ -10168,10 +10171,10 @@
         <v>154</v>
       </c>
       <c r="B15" s="69" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="16">
@@ -10179,21 +10182,21 @@
         <v>160</v>
       </c>
       <c r="B16" s="69" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="B17" s="69" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="18">
@@ -10201,10 +10204,10 @@
         <v>142</v>
       </c>
       <c r="B18" s="69" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="19">
@@ -10212,21 +10215,21 @@
         <v>156</v>
       </c>
       <c r="B19" s="69" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="B20" s="69" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="21">
@@ -10234,10 +10237,10 @@
         <v>151</v>
       </c>
       <c r="B21" s="69" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="22">
@@ -10245,21 +10248,21 @@
         <v>155</v>
       </c>
       <c r="B22" s="69" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="B23" s="69" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="24">
@@ -10267,10 +10270,10 @@
         <v>153</v>
       </c>
       <c r="B24" s="69" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="25">
@@ -10278,10 +10281,10 @@
         <v>198</v>
       </c>
       <c r="B25" s="69" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
   </sheetData>
@@ -20294,7 +20297,7 @@
         <v>22</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>25</v>
+        <v>268</v>
       </c>
       <c r="C7" s="15" t="s">
         <v>26</v>
@@ -23010,7 +23013,7 @@
         <v>42</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C14" s="15" t="s">
         <v>44</v>
@@ -23783,7 +23786,7 @@
     </row>
     <row r="18">
       <c r="DP18" s="1" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
spa recap and projections fix
</commit_message>
<xml_diff>
--- a/the_alternative_f1/The_Alternative_F1.xlsx
+++ b/the_alternative_f1/The_Alternative_F1.xlsx
@@ -1713,10 +1713,10 @@
     <xf borderId="8" fillId="8" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="right" vertical="bottom"/>
     </xf>
-    <xf borderId="4" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="5" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
     <xf borderId="8" fillId="8" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
@@ -3486,9 +3486,13 @@
         <f>IFERROR((VLOOKUP(AJ2,Scoring!$A:$B,2,0))+IF(AM2="y",1,0)+IF(AN2="y",1,0)+IF(AO2="y",1,0)+IF(AP2="y",1,0),0)</f>
         <v>15</v>
       </c>
-      <c r="AR2" s="86"/>
-      <c r="AS2" s="87"/>
-      <c r="AT2" s="87"/>
+      <c r="AR2" s="79">
+        <v>1.0</v>
+      </c>
+      <c r="AS2" s="80">
+        <v>3.0</v>
+      </c>
+      <c r="AT2" s="86"/>
       <c r="AU2" s="81" t="s">
         <v>129</v>
       </c>
@@ -3503,10 +3507,14 @@
       </c>
       <c r="AY2" s="85">
         <f>IFERROR((VLOOKUP(AR2,Scoring!$D:$E,2,0))+IF(AU2="y",1,0)+IF(AV2="y",1,0)+IF(AW2="y",1,0)+IF(AX2="y",1,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="AZ2" s="16"/>
-      <c r="BA2" s="17"/>
+        <v>8</v>
+      </c>
+      <c r="AZ2" s="16">
+        <v>2.0</v>
+      </c>
+      <c r="BA2" s="17">
+        <v>9.0</v>
+      </c>
       <c r="BB2" s="17"/>
       <c r="BC2" s="18" t="s">
         <v>129</v>
@@ -3515,14 +3523,14 @@
         <v>129</v>
       </c>
       <c r="BE2" s="20" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="BF2" s="21" t="s">
         <v>129</v>
       </c>
       <c r="BG2" s="78">
         <f>IFERROR((VLOOKUP(AZ2,Scoring!$A:$B,2,0))+IF(BC2="y",1,0)+IF(BD2="y",1,0)+IF(BE2="y",1,0)+IF(BF2="y",1,0),0)</f>
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="BH2" s="16"/>
       <c r="BI2" s="17"/>
@@ -3543,9 +3551,9 @@
         <f>IFERROR((VLOOKUP(BH2,Scoring!$A:$B,2,0))+IF(BK2="y",1,0)+IF(BL2="y",1,0)+IF(BM2="y",1,0)+IF(BN2="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="BP2" s="86"/>
-      <c r="BQ2" s="87"/>
-      <c r="BR2" s="87"/>
+      <c r="BP2" s="87"/>
+      <c r="BQ2" s="86"/>
+      <c r="BR2" s="86"/>
       <c r="BS2" s="81" t="s">
         <v>129</v>
       </c>
@@ -3619,9 +3627,9 @@
         <f>IFERROR((VLOOKUP(CN2,Scoring!$A:$B,2,0))+IF(CQ2="y",1,0)+IF(CR2="y",1,0)+IF(CS2="y",1,0)+IF(CT2="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="CV2" s="86"/>
-      <c r="CW2" s="87"/>
-      <c r="CX2" s="87"/>
+      <c r="CV2" s="87"/>
+      <c r="CW2" s="86"/>
+      <c r="CX2" s="86"/>
       <c r="CY2" s="81" t="s">
         <v>129</v>
       </c>
@@ -3676,9 +3684,9 @@
         <f>IFERROR((VLOOKUP(DL2,Scoring!$A:$B,2,0))+IF(DO2="y",1,0)+IF(DP2="y",1,0)+IF(DQ2="y",1,0)+IF(DR2="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="DT2" s="86"/>
-      <c r="DU2" s="87"/>
-      <c r="DV2" s="87"/>
+      <c r="DT2" s="87"/>
+      <c r="DU2" s="86"/>
+      <c r="DV2" s="86"/>
       <c r="DW2" s="81" t="s">
         <v>129</v>
       </c>
@@ -3902,8 +3910,12 @@
         <f>IFERROR((VLOOKUP(AJ3,Scoring!$A:$B,2,0))+IF(AM3="y",1,0)+IF(AN3="y",1,0)+IF(AO3="y",1,0)+IF(AP3="y",1,0),0)</f>
         <v>4</v>
       </c>
-      <c r="AR3" s="103"/>
-      <c r="AS3" s="98"/>
+      <c r="AR3" s="96">
+        <v>23.0</v>
+      </c>
+      <c r="AS3" s="97">
+        <v>6.0</v>
+      </c>
       <c r="AT3" s="98"/>
       <c r="AU3" s="99" t="s">
         <v>129</v>
@@ -3921,8 +3933,12 @@
         <f>IFERROR((VLOOKUP(AR3,Scoring!$D:$E,2,0))+IF(AU3="y",1,0)+IF(AV3="y",1,0)+IF(AW3="y",1,0)+IF(AX3="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="AZ3" s="24"/>
-      <c r="BA3" s="25"/>
+      <c r="AZ3" s="24">
+        <v>24.0</v>
+      </c>
+      <c r="BA3" s="25">
+        <v>24.0</v>
+      </c>
       <c r="BB3" s="25"/>
       <c r="BC3" s="26" t="s">
         <v>129</v>
@@ -4316,8 +4332,12 @@
         <f>IFERROR((VLOOKUP(AJ4,Scoring!$A:$B,2,0))+IF(AM4="y",1,0)+IF(AN4="y",1,0)+IF(AO4="y",1,0)+IF(AP4="y",1,0),0)</f>
         <v>12</v>
       </c>
-      <c r="AR4" s="118"/>
-      <c r="AS4" s="113"/>
+      <c r="AR4" s="111">
+        <v>2.0</v>
+      </c>
+      <c r="AS4" s="112">
+        <v>1.0</v>
+      </c>
       <c r="AT4" s="113"/>
       <c r="AU4" s="114" t="s">
         <v>129</v>
@@ -4333,10 +4353,14 @@
       </c>
       <c r="AY4" s="85">
         <f>IFERROR((VLOOKUP(AR4,Scoring!$D:$E,2,0))+IF(AU4="y",1,0)+IF(AV4="y",1,0)+IF(AW4="y",1,0)+IF(AX4="y",1,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="AZ4" s="36"/>
-      <c r="BA4" s="37"/>
+        <v>7</v>
+      </c>
+      <c r="AZ4" s="36">
+        <v>4.0</v>
+      </c>
+      <c r="BA4" s="37">
+        <v>8.0</v>
+      </c>
       <c r="BB4" s="37"/>
       <c r="BC4" s="38" t="s">
         <v>129</v>
@@ -4348,11 +4372,11 @@
         <v>129</v>
       </c>
       <c r="BF4" s="41" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="BG4" s="78">
         <f>IFERROR((VLOOKUP(AZ4,Scoring!$A:$B,2,0))+IF(BC4="y",1,0)+IF(BD4="y",1,0)+IF(BE4="y",1,0)+IF(BF4="y",1,0),0)</f>
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="BH4" s="36"/>
       <c r="BI4" s="37"/>
@@ -4736,9 +4760,15 @@
         <f>IFERROR((VLOOKUP(AJ5,Scoring!$A:$B,2,0))+IF(AM5="y",1,0)+IF(AN5="y",1,0)+IF(AO5="y",1,0)+IF(AP5="y",1,0),0)</f>
         <v>11</v>
       </c>
-      <c r="AR5" s="132"/>
-      <c r="AS5" s="127"/>
-      <c r="AT5" s="127"/>
+      <c r="AR5" s="125">
+        <v>5.0</v>
+      </c>
+      <c r="AS5" s="126">
+        <v>24.0</v>
+      </c>
+      <c r="AT5" s="126">
+        <v>10.0</v>
+      </c>
       <c r="AU5" s="128" t="s">
         <v>129</v>
       </c>
@@ -4753,10 +4783,14 @@
       </c>
       <c r="AY5" s="85">
         <f>IFERROR((VLOOKUP(AR5,Scoring!$D:$E,2,0))+IF(AU5="y",1,0)+IF(AV5="y",1,0)+IF(AW5="y",1,0)+IF(AX5="y",1,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="AZ5" s="48"/>
-      <c r="BA5" s="49"/>
+        <v>4</v>
+      </c>
+      <c r="AZ5" s="48">
+        <v>23.0</v>
+      </c>
+      <c r="BA5" s="49">
+        <v>5.0</v>
+      </c>
       <c r="BB5" s="49"/>
       <c r="BC5" s="50" t="s">
         <v>129</v>
@@ -5150,8 +5184,12 @@
         <f>IFERROR((VLOOKUP(AJ6,Scoring!$A:$B,2,0))+IF(AM6="y",1,0)+IF(AN6="y",1,0)+IF(AO6="y",1,0)+IF(AP6="y",1,0),0)</f>
         <v>4</v>
       </c>
-      <c r="AR6" s="103"/>
-      <c r="AS6" s="98"/>
+      <c r="AR6" s="96">
+        <v>4.0</v>
+      </c>
+      <c r="AS6" s="97">
+        <v>2.0</v>
+      </c>
       <c r="AT6" s="98"/>
       <c r="AU6" s="99" t="s">
         <v>129</v>
@@ -5167,10 +5205,14 @@
       </c>
       <c r="AY6" s="85">
         <f>IFERROR((VLOOKUP(AR6,Scoring!$D:$E,2,0))+IF(AU6="y",1,0)+IF(AV6="y",1,0)+IF(AW6="y",1,0)+IF(AX6="y",1,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="AZ6" s="24"/>
-      <c r="BA6" s="25"/>
+        <v>5</v>
+      </c>
+      <c r="AZ6" s="24">
+        <v>5.0</v>
+      </c>
+      <c r="BA6" s="25">
+        <v>6.0</v>
+      </c>
       <c r="BB6" s="25"/>
       <c r="BC6" s="26" t="s">
         <v>129</v>
@@ -5186,7 +5228,7 @@
       </c>
       <c r="BG6" s="78">
         <f>IFERROR((VLOOKUP(AZ6,Scoring!$A:$B,2,0))+IF(BC6="y",1,0)+IF(BD6="y",1,0)+IF(BE6="y",1,0)+IF(BF6="y",1,0),0)</f>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="BH6" s="24"/>
       <c r="BI6" s="25"/>
@@ -5564,8 +5606,12 @@
         <f>IFERROR((VLOOKUP(AJ7,Scoring!$A:$B,2,0))+IF(AM7="y",1,0)+IF(AN7="y",1,0)+IF(AO7="y",1,0)+IF(AP7="y",1,0),0)</f>
         <v>26</v>
       </c>
-      <c r="AR7" s="103"/>
-      <c r="AS7" s="98"/>
+      <c r="AR7" s="96">
+        <v>23.0</v>
+      </c>
+      <c r="AS7" s="97">
+        <v>5.0</v>
+      </c>
       <c r="AT7" s="98"/>
       <c r="AU7" s="99" t="s">
         <v>129</v>
@@ -5583,11 +5629,15 @@
         <f>IFERROR((VLOOKUP(AR7,Scoring!$D:$E,2,0))+IF(AU7="y",1,0)+IF(AV7="y",1,0)+IF(AW7="y",1,0)+IF(AX7="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="AZ7" s="24"/>
-      <c r="BA7" s="25"/>
+      <c r="AZ7" s="24">
+        <v>8.0</v>
+      </c>
+      <c r="BA7" s="25">
+        <v>10.0</v>
+      </c>
       <c r="BB7" s="25"/>
       <c r="BC7" s="26" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="BD7" s="27" t="s">
         <v>129</v>
@@ -5600,7 +5650,7 @@
       </c>
       <c r="BG7" s="95">
         <f>IFERROR((VLOOKUP(AZ7,Scoring!$A:$B,2,0))+IF(BC7="y",1,0)+IF(BD7="y",1,0)+IF(BE7="y",1,0)+IF(BF7="y",1,0),0)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="BH7" s="24"/>
       <c r="BI7" s="25"/>
@@ -5978,8 +6028,12 @@
         <f>IFERROR((VLOOKUP(AJ8,Scoring!$A:$B,2,0))+IF(AM8="y",1,0)+IF(AN8="y",1,0)+IF(AO8="y",1,0)+IF(AP8="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="AR8" s="118"/>
-      <c r="AS8" s="113"/>
+      <c r="AR8" s="111">
+        <v>8.0</v>
+      </c>
+      <c r="AS8" s="112">
+        <v>8.0</v>
+      </c>
       <c r="AT8" s="113"/>
       <c r="AU8" s="114" t="s">
         <v>129</v>
@@ -5995,10 +6049,14 @@
       </c>
       <c r="AY8" s="85">
         <f>IFERROR((VLOOKUP(AR8,Scoring!$D:$E,2,0))+IF(AU8="y",1,0)+IF(AV8="y",1,0)+IF(AW8="y",1,0)+IF(AX8="y",1,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="AZ8" s="36"/>
-      <c r="BA8" s="37"/>
+        <v>1</v>
+      </c>
+      <c r="AZ8" s="36">
+        <v>9.0</v>
+      </c>
+      <c r="BA8" s="37">
+        <v>2.0</v>
+      </c>
       <c r="BB8" s="37"/>
       <c r="BC8" s="38" t="s">
         <v>129</v>
@@ -6014,7 +6072,7 @@
       </c>
       <c r="BG8" s="78">
         <f>IFERROR((VLOOKUP(AZ8,Scoring!$A:$B,2,0))+IF(BC8="y",1,0)+IF(BD8="y",1,0)+IF(BE8="y",1,0)+IF(BF8="y",1,0),0)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="BH8" s="36"/>
       <c r="BI8" s="37"/>
@@ -6392,8 +6450,12 @@
         <f>IFERROR((VLOOKUP(AJ9,Scoring!$A:$B,2,0))+IF(AM9="y",1,0)+IF(AN9="y",1,0)+IF(AO9="y",1,0)+IF(AP9="y",1,0),0)</f>
         <v>2</v>
       </c>
-      <c r="AR9" s="132"/>
-      <c r="AS9" s="127"/>
+      <c r="AR9" s="125">
+        <v>7.0</v>
+      </c>
+      <c r="AS9" s="126">
+        <v>9.0</v>
+      </c>
       <c r="AT9" s="127"/>
       <c r="AU9" s="128" t="s">
         <v>129</v>
@@ -6409,10 +6471,14 @@
       </c>
       <c r="AY9" s="85">
         <f>IFERROR((VLOOKUP(AR9,Scoring!$D:$E,2,0))+IF(AU9="y",1,0)+IF(AV9="y",1,0)+IF(AW9="y",1,0)+IF(AX9="y",1,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="AZ9" s="48"/>
-      <c r="BA9" s="49"/>
+        <v>2</v>
+      </c>
+      <c r="AZ9" s="48">
+        <v>3.0</v>
+      </c>
+      <c r="BA9" s="49">
+        <v>3.0</v>
+      </c>
       <c r="BB9" s="49"/>
       <c r="BC9" s="50" t="s">
         <v>129</v>
@@ -6428,7 +6494,7 @@
       </c>
       <c r="BG9" s="95">
         <f>IFERROR((VLOOKUP(AZ9,Scoring!$A:$B,2,0))+IF(BC9="y",1,0)+IF(BD9="y",1,0)+IF(BE9="y",1,0)+IF(BF9="y",1,0),0)</f>
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="BH9" s="48"/>
       <c r="BI9" s="49"/>
@@ -6806,8 +6872,12 @@
         <f>IFERROR((VLOOKUP(AJ10,Scoring!$A:$B,2,0))+IF(AM10="y",1,0)+IF(AN10="y",1,0)+IF(AO10="y",1,0)+IF(AP10="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="AR10" s="103"/>
-      <c r="AS10" s="98"/>
+      <c r="AR10" s="96">
+        <v>24.0</v>
+      </c>
+      <c r="AS10" s="97">
+        <v>24.0</v>
+      </c>
       <c r="AT10" s="98"/>
       <c r="AU10" s="99" t="s">
         <v>129</v>
@@ -6825,8 +6895,12 @@
         <f>IFERROR((VLOOKUP(AR10,Scoring!$D:$E,2,0))+IF(AU10="y",1,0)+IF(AV10="y",1,0)+IF(AW10="y",1,0)+IF(AX10="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="AZ10" s="24"/>
-      <c r="BA10" s="25"/>
+      <c r="AZ10" s="24">
+        <v>24.0</v>
+      </c>
+      <c r="BA10" s="25">
+        <v>24.0</v>
+      </c>
       <c r="BB10" s="25"/>
       <c r="BC10" s="26" t="s">
         <v>129</v>
@@ -7220,8 +7294,12 @@
         <f>IFERROR((VLOOKUP(AJ11,Scoring!$A:$B,2,0))+IF(AM11="y",1,0)+IF(AN11="y",1,0)+IF(AO11="y",1,0)+IF(AP11="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="AR11" s="103"/>
-      <c r="AS11" s="98"/>
+      <c r="AR11" s="96">
+        <v>24.0</v>
+      </c>
+      <c r="AS11" s="97">
+        <v>24.0</v>
+      </c>
       <c r="AT11" s="98"/>
       <c r="AU11" s="99" t="s">
         <v>129</v>
@@ -7239,8 +7317,12 @@
         <f>IFERROR((VLOOKUP(AR11,Scoring!$D:$E,2,0))+IF(AU11="y",1,0)+IF(AV11="y",1,0)+IF(AW11="y",1,0)+IF(AX11="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="AZ11" s="24"/>
-      <c r="BA11" s="25"/>
+      <c r="AZ11" s="24">
+        <v>24.0</v>
+      </c>
+      <c r="BA11" s="25">
+        <v>24.0</v>
+      </c>
       <c r="BB11" s="25"/>
       <c r="BC11" s="26" t="s">
         <v>129</v>
@@ -7634,8 +7716,12 @@
         <f>IFERROR((VLOOKUP(AJ12,Scoring!$A:$B,2,0))+IF(AM12="y",1,0)+IF(AN12="y",1,0)+IF(AO12="y",1,0)+IF(AP12="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="AR12" s="118"/>
-      <c r="AS12" s="113"/>
+      <c r="AR12" s="111">
+        <v>24.0</v>
+      </c>
+      <c r="AS12" s="112">
+        <v>24.0</v>
+      </c>
       <c r="AT12" s="113"/>
       <c r="AU12" s="114" t="s">
         <v>129</v>
@@ -7653,8 +7739,12 @@
         <f>IFERROR((VLOOKUP(AR12,Scoring!$D:$E,2,0))+IF(AU12="y",1,0)+IF(AV12="y",1,0)+IF(AW12="y",1,0)+IF(AX12="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="AZ12" s="36"/>
-      <c r="BA12" s="37"/>
+      <c r="AZ12" s="36">
+        <v>24.0</v>
+      </c>
+      <c r="BA12" s="37">
+        <v>24.0</v>
+      </c>
       <c r="BB12" s="37"/>
       <c r="BC12" s="38" t="s">
         <v>129</v>
@@ -8048,8 +8138,12 @@
         <f>IFERROR((VLOOKUP(AJ13,Scoring!$A:$B,2,0))+IF(AM13="y",1,0)+IF(AN13="y",1,0)+IF(AO13="y",1,0)+IF(AP13="y",1,0),0)</f>
         <v>1</v>
       </c>
-      <c r="AR13" s="103"/>
-      <c r="AS13" s="98"/>
+      <c r="AR13" s="96">
+        <v>9.0</v>
+      </c>
+      <c r="AS13" s="97">
+        <v>7.0</v>
+      </c>
       <c r="AT13" s="98"/>
       <c r="AU13" s="99" t="s">
         <v>129</v>
@@ -8065,10 +8159,14 @@
       </c>
       <c r="AY13" s="85">
         <f>IFERROR((VLOOKUP(AR13,Scoring!$D:$E,2,0))+IF(AU13="y",1,0)+IF(AV13="y",1,0)+IF(AW13="y",1,0)+IF(AX13="y",1,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="AZ13" s="24"/>
-      <c r="BA13" s="25"/>
+        <v>0.5</v>
+      </c>
+      <c r="AZ13" s="24">
+        <v>10.0</v>
+      </c>
+      <c r="BA13" s="25">
+        <v>1.0</v>
+      </c>
       <c r="BB13" s="25"/>
       <c r="BC13" s="26" t="s">
         <v>129</v>
@@ -8084,7 +8182,7 @@
       </c>
       <c r="BG13" s="95">
         <f>IFERROR((VLOOKUP(AZ13,Scoring!$A:$B,2,0))+IF(BC13="y",1,0)+IF(BD13="y",1,0)+IF(BE13="y",1,0)+IF(BF13="y",1,0),0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BH13" s="24"/>
       <c r="BI13" s="25"/>
@@ -8462,9 +8560,15 @@
         <f>IFERROR((VLOOKUP(AJ14,Scoring!$A:$B,2,0))+IF(AM14="y",1,0)+IF(AN14="y",1,0)+IF(AO14="y",1,0)+IF(AP14="y",1,0),0)</f>
         <v>18</v>
       </c>
-      <c r="AR14" s="118"/>
-      <c r="AS14" s="113"/>
-      <c r="AT14" s="113"/>
+      <c r="AR14" s="111">
+        <v>3.0</v>
+      </c>
+      <c r="AS14" s="112">
+        <v>24.0</v>
+      </c>
+      <c r="AT14" s="112">
+        <v>11.0</v>
+      </c>
       <c r="AU14" s="114" t="s">
         <v>129</v>
       </c>
@@ -8479,10 +8583,14 @@
       </c>
       <c r="AY14" s="85">
         <f>IFERROR((VLOOKUP(AR14,Scoring!$D:$E,2,0))+IF(AU14="y",1,0)+IF(AV14="y",1,0)+IF(AW14="y",1,0)+IF(AX14="y",1,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="AZ14" s="36"/>
-      <c r="BA14" s="37"/>
+        <v>6</v>
+      </c>
+      <c r="AZ14" s="36">
+        <v>6.0</v>
+      </c>
+      <c r="BA14" s="37">
+        <v>7.0</v>
+      </c>
       <c r="BB14" s="37"/>
       <c r="BC14" s="38" t="s">
         <v>129</v>
@@ -8498,7 +8606,7 @@
       </c>
       <c r="BG14" s="78">
         <f>IFERROR((VLOOKUP(AZ14,Scoring!$A:$B,2,0))+IF(BC14="y",1,0)+IF(BD14="y",1,0)+IF(BE14="y",1,0)+IF(BF14="y",1,0),0)</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="BH14" s="36"/>
       <c r="BI14" s="37"/>
@@ -8878,8 +8986,12 @@
         <f>IFERROR((VLOOKUP(AJ15,Scoring!$A:$B,2,0))+IF(AM15="y",1,0)+IF(AN15="y",1,0)+IF(AO15="y",1,0)+IF(AP15="y",1,0),0)</f>
         <v>9</v>
       </c>
-      <c r="AR15" s="132"/>
-      <c r="AS15" s="127"/>
+      <c r="AR15" s="125">
+        <v>7.0</v>
+      </c>
+      <c r="AS15" s="126">
+        <v>4.0</v>
+      </c>
       <c r="AT15" s="127"/>
       <c r="AU15" s="128" t="s">
         <v>129</v>
@@ -8895,10 +9007,14 @@
       </c>
       <c r="AY15" s="85">
         <f>IFERROR((VLOOKUP(AR15,Scoring!$D:$E,2,0))+IF(AU15="y",1,0)+IF(AV15="y",1,0)+IF(AW15="y",1,0)+IF(AX15="y",1,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="AZ15" s="48"/>
-      <c r="BA15" s="49"/>
+        <v>2</v>
+      </c>
+      <c r="AZ15" s="48">
+        <v>1.0</v>
+      </c>
+      <c r="BA15" s="49">
+        <v>4.0</v>
+      </c>
       <c r="BB15" s="49"/>
       <c r="BC15" s="50" t="s">
         <v>129</v>
@@ -8914,7 +9030,7 @@
       </c>
       <c r="BG15" s="95">
         <f>IFERROR((VLOOKUP(AZ15,Scoring!$A:$B,2,0))+IF(BC15="y",1,0)+IF(BD15="y",1,0)+IF(BE15="y",1,0)+IF(BF15="y",1,0),0)</f>
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="BH15" s="48"/>
       <c r="BI15" s="49"/>
@@ -9292,9 +9408,15 @@
         <f>IFERROR((VLOOKUP(AJ16,Scoring!$A:$B,2,0))+IF(AM16="y",1,0)+IF(AN16="y",1,0)+IF(AO16="y",1,0)+IF(AP16="y",1,0),0)</f>
         <v>6</v>
       </c>
-      <c r="AR16" s="103"/>
-      <c r="AS16" s="98"/>
-      <c r="AT16" s="98"/>
+      <c r="AR16" s="96">
+        <v>25.0</v>
+      </c>
+      <c r="AS16" s="97">
+        <v>24.0</v>
+      </c>
+      <c r="AT16" s="97">
+        <v>12.0</v>
+      </c>
       <c r="AU16" s="99" t="s">
         <v>129</v>
       </c>
@@ -9311,14 +9433,18 @@
         <f>IFERROR((VLOOKUP(AR16,Scoring!$D:$E,2,0))+IF(AU16="y",1,0)+IF(AV16="y",1,0)+IF(AW16="y",1,0)+IF(AX16="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="AZ16" s="24"/>
-      <c r="BA16" s="25"/>
+      <c r="AZ16" s="24">
+        <v>7.0</v>
+      </c>
+      <c r="BA16" s="25">
+        <v>11.0</v>
+      </c>
       <c r="BB16" s="25"/>
       <c r="BC16" s="26" t="s">
         <v>129</v>
       </c>
       <c r="BD16" s="27" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="BE16" s="28" t="s">
         <v>129</v>
@@ -9328,7 +9454,7 @@
       </c>
       <c r="BG16" s="78">
         <f>IFERROR((VLOOKUP(AZ16,Scoring!$A:$B,2,0))+IF(BC16="y",1,0)+IF(BD16="y",1,0)+IF(BE16="y",1,0)+IF(BF16="y",1,0),0)</f>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="BH16" s="24"/>
       <c r="BI16" s="25"/>
@@ -9708,8 +9834,12 @@
         <f>IFERROR((VLOOKUP(AJ17,Scoring!$A:$B,2,0))+IF(AM17="y",1,0)+IF(AN17="y",1,0)+IF(AO17="y",1,0)+IF(AP17="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="AR17" s="147"/>
-      <c r="AS17" s="142"/>
+      <c r="AR17" s="140">
+        <v>24.0</v>
+      </c>
+      <c r="AS17" s="141">
+        <v>24.0</v>
+      </c>
       <c r="AT17" s="142"/>
       <c r="AU17" s="143" t="s">
         <v>129</v>
@@ -9727,8 +9857,12 @@
         <f>IFERROR((VLOOKUP(AR17,Scoring!$D:$E,2,0))+IF(AU17="y",1,0)+IF(AV17="y",1,0)+IF(AW17="y",1,0)+IF(AX17="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="AZ17" s="60"/>
-      <c r="BA17" s="61"/>
+      <c r="AZ17" s="60">
+        <v>24.0</v>
+      </c>
+      <c r="BA17" s="61">
+        <v>24.0</v>
+      </c>
       <c r="BB17" s="61"/>
       <c r="BC17" s="62" t="s">
         <v>129</v>

</xml_diff>